<commit_message>
Adjust With latest plan
</commit_message>
<xml_diff>
--- a/public/docs/Template_Shikake_Bonder.xlsx
+++ b/public/docs/Template_Shikake_Bonder.xlsx
@@ -1,26 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29426"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr codeName="ThisWorkbook"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Code\laragon\www\jai_ekanban\public\docs\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87A6044C-193C-4ECE-8072-05F6166D67E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17790" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView activeTab="0" autoFilterDateGrouping="true" firstSheet="0" minimized="false" showHorizontalScroll="true" showSheetTabs="true" showVerticalScroll="true" tabRatio="600" visibility="visible"/>
   </bookViews>
   <sheets>
-    <sheet name="Data" sheetId="1" r:id="rId1"/>
+    <sheet name="Data" sheetId="1" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <definedNames/>
+  <calcPr calcId="999999" calcMode="auto" calcCompleted="1" fullCalcOnLoad="0" forceFullCalc="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="44">
+  <si>
+    <t>Carline</t>
+  </si>
   <si>
     <t>Conveyor</t>
   </si>
@@ -34,12 +32,12 @@
     <t>Family</t>
   </si>
   <si>
+    <t>Sequence</t>
+  </si>
+  <si>
     <t>Released Note</t>
   </si>
   <si>
-    <t>Sequence</t>
-  </si>
-  <si>
     <t>Bonder No</t>
   </si>
   <si>
@@ -142,27 +140,50 @@
     <t>Bonder No B 7</t>
   </si>
   <si>
-    <t>Carline</t>
+    <t>ASSY-001</t>
+  </si>
+  <si>
+    <t>ASSY-002</t>
+  </si>
+  <si>
+    <t>ASSY-003</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="3">
     <font>
+      <b val="0"/>
+      <i val="0"/>
+      <strike val="0"/>
+      <u val="none"/>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
     </font>
     <font>
-      <b/>
+      <b val="1"/>
+      <i val="0"/>
+      <strike val="0"/>
+      <u val="none"/>
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
     </font>
+    <font>
+      <b val="1"/>
+      <i val="1"/>
+      <strike val="0"/>
+      <u val="none"/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -172,6 +193,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF4472C4"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
         <bgColor rgb="FF000000"/>
       </patternFill>
     </fill>
@@ -203,25 +230,20 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+  <cellXfs count="3">
+    <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
+    <xf xfId="0" fontId="1" numFmtId="0" fillId="2" borderId="1" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="2" numFmtId="0" fillId="3" borderId="1" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <tableStyles defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotTableStyle1"/>
 </styleSheet>
 </file>
 
@@ -511,178 +533,196 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AO1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+  </sheetPr>
+  <dimension ref="A1:AR1"/>
+  <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="2" max="2" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="6.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="18.7109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="14" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="8.140625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="15.140625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="22.28515625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="21" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="15.140625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="18.7109375" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="15.140625" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="18.7109375" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="15.140625" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="18.7109375" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="15.140625" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="18.7109375" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="15.140625" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="18.7109375" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="15.140625" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="18.7109375" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="15.140625" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="18.7109375" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="15.140625" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="18.7109375" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="15.140625" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="18.7109375" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="15.140625" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="18.7109375" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="15.140625" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="18.7109375" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="15.140625" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="18.7109375" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="15.140625" bestFit="1" customWidth="1"/>
-    <col min="39" max="39" width="18.7109375" bestFit="1" customWidth="1"/>
-    <col min="40" max="40" width="15.140625" bestFit="1" customWidth="1"/>
-    <col min="41" max="41" width="18.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.569" bestFit="true" customWidth="true" style="0"/>
+    <col min="2" max="2" width="12.854" bestFit="true" customWidth="true" style="0"/>
+    <col min="3" max="3" width="11.569" bestFit="true" customWidth="true" style="0"/>
+    <col min="4" max="4" width="6.856" bestFit="true" customWidth="true" style="0"/>
+    <col min="5" max="5" width="10.426" bestFit="true" customWidth="true" style="0"/>
+    <col min="6" max="6" width="12.854" bestFit="true" customWidth="true" style="0"/>
+    <col min="7" max="7" width="18.71" bestFit="true" customWidth="true" style="0"/>
+    <col min="8" max="8" width="13.997" bestFit="true" customWidth="true" style="0"/>
+    <col min="9" max="9" width="11.569" bestFit="true" customWidth="true" style="0"/>
+    <col min="10" max="10" width="8.141" bestFit="true" customWidth="true" style="0"/>
+    <col min="11" max="11" width="15.139" bestFit="true" customWidth="true" style="0"/>
+    <col min="12" max="12" width="22.28" bestFit="true" customWidth="true" style="0"/>
+    <col min="13" max="13" width="20.995" bestFit="true" customWidth="true" style="0"/>
+    <col min="14" max="14" width="15.139" bestFit="true" customWidth="true" style="0"/>
+    <col min="15" max="15" width="18.71" bestFit="true" customWidth="true" style="0"/>
+    <col min="16" max="16" width="15.139" bestFit="true" customWidth="true" style="0"/>
+    <col min="17" max="17" width="18.71" bestFit="true" customWidth="true" style="0"/>
+    <col min="18" max="18" width="15.139" bestFit="true" customWidth="true" style="0"/>
+    <col min="19" max="19" width="18.71" bestFit="true" customWidth="true" style="0"/>
+    <col min="20" max="20" width="15.139" bestFit="true" customWidth="true" style="0"/>
+    <col min="21" max="21" width="18.71" bestFit="true" customWidth="true" style="0"/>
+    <col min="22" max="22" width="15.139" bestFit="true" customWidth="true" style="0"/>
+    <col min="23" max="23" width="18.71" bestFit="true" customWidth="true" style="0"/>
+    <col min="24" max="24" width="15.139" bestFit="true" customWidth="true" style="0"/>
+    <col min="25" max="25" width="18.71" bestFit="true" customWidth="true" style="0"/>
+    <col min="26" max="26" width="15.139" bestFit="true" customWidth="true" style="0"/>
+    <col min="27" max="27" width="18.71" bestFit="true" customWidth="true" style="0"/>
+    <col min="28" max="28" width="15.139" bestFit="true" customWidth="true" style="0"/>
+    <col min="29" max="29" width="18.71" bestFit="true" customWidth="true" style="0"/>
+    <col min="30" max="30" width="15.139" bestFit="true" customWidth="true" style="0"/>
+    <col min="31" max="31" width="18.71" bestFit="true" customWidth="true" style="0"/>
+    <col min="32" max="32" width="15.139" bestFit="true" customWidth="true" style="0"/>
+    <col min="33" max="33" width="18.71" bestFit="true" customWidth="true" style="0"/>
+    <col min="34" max="34" width="15.139" bestFit="true" customWidth="true" style="0"/>
+    <col min="35" max="35" width="18.71" bestFit="true" customWidth="true" style="0"/>
+    <col min="36" max="36" width="15.139" bestFit="true" customWidth="true" style="0"/>
+    <col min="37" max="37" width="18.71" bestFit="true" customWidth="true" style="0"/>
+    <col min="38" max="38" width="15.139" bestFit="true" customWidth="true" style="0"/>
+    <col min="39" max="39" width="18.71" bestFit="true" customWidth="true" style="0"/>
+    <col min="40" max="40" width="15.139" bestFit="true" customWidth="true" style="0"/>
+    <col min="41" max="41" width="18.71" bestFit="true" customWidth="true" style="0"/>
+    <col min="42" max="42" width="12.854" bestFit="true" customWidth="true" style="0"/>
+    <col min="43" max="43" width="12.854" bestFit="true" customWidth="true" style="0"/>
+    <col min="44" max="44" width="12.854" bestFit="true" customWidth="true" style="0"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:41" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:44">
       <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="R1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="S1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="T1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="U1" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="V1" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="W1" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="X1" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="Y1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="Z1" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="AA1" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="AB1" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="AC1" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="AD1" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="AE1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="AF1" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="AG1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="AH1" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="AI1" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="AJ1" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="AK1" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="AL1" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="AM1" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="AN1" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="AO1" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="N1" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="O1" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="P1" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="Q1" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="R1" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="S1" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="T1" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="U1" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="V1" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="W1" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="X1" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="Y1" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="Z1" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="AA1" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="AB1" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="AC1" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="AD1" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="AE1" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="AF1" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="AG1" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="AH1" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="AI1" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="AJ1" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="AK1" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="AL1" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="AM1" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="AN1" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="AO1" s="1" t="s">
-        <v>39</v>
+      <c r="AP1" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="AQ1" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="AR1" s="2" t="s">
+        <v>43</v>
       </c>
     </row>
   </sheetData>
+  <printOptions gridLines="false" gridLinesSet="true"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="1" orientation="default" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix: correct getAssyStartColumn and regenerate shikake templates with QRCode Drawing
</commit_message>
<xml_diff>
--- a/public/docs/Template_Shikake_Bonder.xlsx
+++ b/public/docs/Template_Shikake_Bonder.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="42">
   <si>
     <t>Carline</t>
   </si>
@@ -56,6 +56,9 @@
     <t>Barcode Process</t>
   </si>
   <si>
+    <t>QRCode Drawing</t>
+  </si>
+  <si>
     <t>CCT No A 1</t>
   </si>
   <si>
@@ -138,15 +141,6 @@
   </si>
   <si>
     <t>Bonder No B 7</t>
-  </si>
-  <si>
-    <t>ASSY-001</t>
-  </si>
-  <si>
-    <t>ASSY-002</t>
-  </si>
-  <si>
-    <t>ASSY-003</t>
   </si>
 </sst>
 </file>
@@ -154,7 +148,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="2">
     <font>
       <b val="0"/>
       <i val="0"/>
@@ -173,17 +167,8 @@
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
     </font>
-    <font>
-      <b val="1"/>
-      <i val="1"/>
-      <strike val="0"/>
-      <u val="none"/>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-    </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -193,12 +178,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF4472C4"/>
-        <bgColor rgb="FF000000"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF92D050"/>
         <bgColor rgb="FF000000"/>
       </patternFill>
     </fill>
@@ -230,12 +209,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
     <xf xfId="0" fontId="1" numFmtId="0" fillId="2" borderId="1" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
-    </xf>
-    <xf xfId="0" fontId="2" numFmtId="0" fillId="3" borderId="1" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
   </cellXfs>
@@ -537,7 +513,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:AR1"/>
+  <dimension ref="A1:AP1"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="11.569" bestFit="true" customWidth="true" style="0"/>
@@ -553,40 +529,38 @@
     <col min="11" max="11" width="15.139" bestFit="true" customWidth="true" style="0"/>
     <col min="12" max="12" width="22.28" bestFit="true" customWidth="true" style="0"/>
     <col min="13" max="13" width="20.995" bestFit="true" customWidth="true" style="0"/>
-    <col min="14" max="14" width="15.139" bestFit="true" customWidth="true" style="0"/>
-    <col min="15" max="15" width="18.71" bestFit="true" customWidth="true" style="0"/>
-    <col min="16" max="16" width="15.139" bestFit="true" customWidth="true" style="0"/>
-    <col min="17" max="17" width="18.71" bestFit="true" customWidth="true" style="0"/>
-    <col min="18" max="18" width="15.139" bestFit="true" customWidth="true" style="0"/>
-    <col min="19" max="19" width="18.71" bestFit="true" customWidth="true" style="0"/>
-    <col min="20" max="20" width="15.139" bestFit="true" customWidth="true" style="0"/>
-    <col min="21" max="21" width="18.71" bestFit="true" customWidth="true" style="0"/>
-    <col min="22" max="22" width="15.139" bestFit="true" customWidth="true" style="0"/>
-    <col min="23" max="23" width="18.71" bestFit="true" customWidth="true" style="0"/>
-    <col min="24" max="24" width="15.139" bestFit="true" customWidth="true" style="0"/>
-    <col min="25" max="25" width="18.71" bestFit="true" customWidth="true" style="0"/>
-    <col min="26" max="26" width="15.139" bestFit="true" customWidth="true" style="0"/>
-    <col min="27" max="27" width="18.71" bestFit="true" customWidth="true" style="0"/>
-    <col min="28" max="28" width="15.139" bestFit="true" customWidth="true" style="0"/>
-    <col min="29" max="29" width="18.71" bestFit="true" customWidth="true" style="0"/>
-    <col min="30" max="30" width="15.139" bestFit="true" customWidth="true" style="0"/>
-    <col min="31" max="31" width="18.71" bestFit="true" customWidth="true" style="0"/>
-    <col min="32" max="32" width="15.139" bestFit="true" customWidth="true" style="0"/>
-    <col min="33" max="33" width="18.71" bestFit="true" customWidth="true" style="0"/>
-    <col min="34" max="34" width="15.139" bestFit="true" customWidth="true" style="0"/>
-    <col min="35" max="35" width="18.71" bestFit="true" customWidth="true" style="0"/>
-    <col min="36" max="36" width="15.139" bestFit="true" customWidth="true" style="0"/>
-    <col min="37" max="37" width="18.71" bestFit="true" customWidth="true" style="0"/>
-    <col min="38" max="38" width="15.139" bestFit="true" customWidth="true" style="0"/>
-    <col min="39" max="39" width="18.71" bestFit="true" customWidth="true" style="0"/>
-    <col min="40" max="40" width="15.139" bestFit="true" customWidth="true" style="0"/>
-    <col min="41" max="41" width="18.71" bestFit="true" customWidth="true" style="0"/>
-    <col min="42" max="42" width="12.854" bestFit="true" customWidth="true" style="0"/>
-    <col min="43" max="43" width="12.854" bestFit="true" customWidth="true" style="0"/>
-    <col min="44" max="44" width="12.854" bestFit="true" customWidth="true" style="0"/>
+    <col min="14" max="14" width="19.852" bestFit="true" customWidth="true" style="0"/>
+    <col min="15" max="15" width="15.139" bestFit="true" customWidth="true" style="0"/>
+    <col min="16" max="16" width="18.71" bestFit="true" customWidth="true" style="0"/>
+    <col min="17" max="17" width="15.139" bestFit="true" customWidth="true" style="0"/>
+    <col min="18" max="18" width="18.71" bestFit="true" customWidth="true" style="0"/>
+    <col min="19" max="19" width="15.139" bestFit="true" customWidth="true" style="0"/>
+    <col min="20" max="20" width="18.71" bestFit="true" customWidth="true" style="0"/>
+    <col min="21" max="21" width="15.139" bestFit="true" customWidth="true" style="0"/>
+    <col min="22" max="22" width="18.71" bestFit="true" customWidth="true" style="0"/>
+    <col min="23" max="23" width="15.139" bestFit="true" customWidth="true" style="0"/>
+    <col min="24" max="24" width="18.71" bestFit="true" customWidth="true" style="0"/>
+    <col min="25" max="25" width="15.139" bestFit="true" customWidth="true" style="0"/>
+    <col min="26" max="26" width="18.71" bestFit="true" customWidth="true" style="0"/>
+    <col min="27" max="27" width="15.139" bestFit="true" customWidth="true" style="0"/>
+    <col min="28" max="28" width="18.71" bestFit="true" customWidth="true" style="0"/>
+    <col min="29" max="29" width="15.139" bestFit="true" customWidth="true" style="0"/>
+    <col min="30" max="30" width="18.71" bestFit="true" customWidth="true" style="0"/>
+    <col min="31" max="31" width="15.139" bestFit="true" customWidth="true" style="0"/>
+    <col min="32" max="32" width="18.71" bestFit="true" customWidth="true" style="0"/>
+    <col min="33" max="33" width="15.139" bestFit="true" customWidth="true" style="0"/>
+    <col min="34" max="34" width="18.71" bestFit="true" customWidth="true" style="0"/>
+    <col min="35" max="35" width="15.139" bestFit="true" customWidth="true" style="0"/>
+    <col min="36" max="36" width="18.71" bestFit="true" customWidth="true" style="0"/>
+    <col min="37" max="37" width="15.139" bestFit="true" customWidth="true" style="0"/>
+    <col min="38" max="38" width="18.71" bestFit="true" customWidth="true" style="0"/>
+    <col min="39" max="39" width="15.139" bestFit="true" customWidth="true" style="0"/>
+    <col min="40" max="40" width="18.71" bestFit="true" customWidth="true" style="0"/>
+    <col min="41" max="41" width="15.139" bestFit="true" customWidth="true" style="0"/>
+    <col min="42" max="42" width="18.71" bestFit="true" customWidth="true" style="0"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:44">
+    <row r="1" spans="1:42">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -710,14 +684,8 @@
       <c r="AO1" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="AP1" s="2" t="s">
+      <c r="AP1" s="1" t="s">
         <v>41</v>
-      </c>
-      <c r="AQ1" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="AR1" s="2" t="s">
-        <v>43</v>
       </c>
     </row>
   </sheetData>

</xml_diff>